<commit_message>
new calc of density mean
</commit_message>
<xml_diff>
--- a/data/01-31-densitySLF.xlsx
+++ b/data/01-31-densitySLF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jille\Documents\Uni\Master-Mechatronik\Masterarbeit\Messung1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jille\Documents\Uni\Master-Mechatronik\Masterarbeit\SMP-SignalProcessing\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E238D63A-1723-4349-B246-824679626845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5D8477D-4B2D-4F31-B017-FBFD9AC4B841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F87BFA84-DB09-4A4E-8E0E-1B2FD7CE4138}"/>
+    <workbookView xWindow="-28905" yWindow="60" windowWidth="14610" windowHeight="15585" xr2:uid="{F87BFA84-DB09-4A4E-8E0E-1B2FD7CE4138}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>snowdepth</t>
   </si>
@@ -44,13 +44,22 @@
     <t>density SLF in kg/m^3</t>
   </si>
   <si>
-    <t xml:space="preserve">density1 </t>
-  </si>
-  <si>
     <t>snowheight</t>
   </si>
   <si>
     <t>mean</t>
+  </si>
+  <si>
+    <t>density1</t>
+  </si>
+  <si>
+    <t>density2</t>
+  </si>
+  <si>
+    <t>density3</t>
+  </si>
+  <si>
+    <t>density4</t>
   </si>
 </sst>
 </file>
@@ -422,27 +431,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F56E685-F6ED-4C83-A160-21E3B800886C}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>0</v>
       </c>
@@ -456,7 +474,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>8</v>
       </c>
@@ -470,7 +488,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>18</v>
       </c>
@@ -484,7 +502,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>28</v>
       </c>
@@ -498,7 +516,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>38</v>
       </c>
@@ -515,7 +533,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>48</v>
       </c>
@@ -529,7 +547,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>58</v>
       </c>
@@ -543,7 +561,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>68</v>
       </c>
@@ -557,7 +575,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>78</v>
       </c>
@@ -571,7 +589,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>88</v>
       </c>
@@ -594,7 +612,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>98</v>
       </c>

</xml_diff>